<commit_message>
4951 - Update Resource Type Import/Export for MOQ Types
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Tests/ActionLogic/Export/LaborTypesAndSpread.xlsx
+++ b/GenBOE/GenBOE.Tests/ActionLogic/Export/LaborTypesAndSpread.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22527"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\Git\genboe\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF5D9862-E213-4160-AAFC-BCBA56549906}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="90" windowWidth="19320" windowHeight="11760"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Labor Types" sheetId="3" r:id="rId1"/>
     <sheet name="Options Lists" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="Clins">'Options Lists'!$E$2</definedName>
+    <definedName name="CLINs">'Options Lists'!$E$2</definedName>
     <definedName name="COST_STYLE">#REF!</definedName>
+    <definedName name="MOQTypes">'Options Lists'!$G$2</definedName>
+    <definedName name="Offload">'Options Lists'!$F$2</definedName>
     <definedName name="PerfOrgs">'Options Lists'!$B$2</definedName>
     <definedName name="Resources">'Options Lists'!$A$2</definedName>
     <definedName name="SpreadCurves">'Options Lists'!$C$2</definedName>
@@ -28,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="21">
   <si>
     <t>Performing Orgs</t>
   </si>
@@ -84,18 +87,23 @@
     <t>CLIN</t>
   </si>
   <si>
-    <t>Reference</t>
+    <t>Offload</t>
+  </si>
+  <si>
+    <t>MOQ Type</t>
+  </si>
+  <si>
+    <t>MOQTypes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/yyyy"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -118,8 +126,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFECF0F1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFECF0F1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF452DB2"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -135,6 +171,36 @@
           <color theme="0" tint="-0.25098422193060094"/>
         </stop>
       </gradientFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF070729"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9F9F9F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF452DB2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD35714"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -157,13 +223,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="8">
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="0"/>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="0"/>
+    <xf numFmtId="49" fontId="3" fillId="5" borderId="0"/>
+    <xf numFmtId="49" fontId="3" fillId="6" borderId="0"/>
+    <xf numFmtId="49" fontId="6" fillId="7" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -171,20 +243,17 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="genBOE" xfId="1"/>
+  <cellStyles count="8">
+    <cellStyle name="genBOE" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
+    <cellStyle name="PPDuplicateRow" xfId="5" xr:uid="{9122EC09-67FD-49C5-95A4-2D9419B3FEE0}"/>
+    <cellStyle name="PPHeaderColumn" xfId="3" xr:uid="{37FD2640-2E85-4306-88DE-A00E421F402E}"/>
+    <cellStyle name="PPHeaderRequired" xfId="4" xr:uid="{180094FB-4A1F-402E-8045-8F1F9F48FF85}"/>
+    <cellStyle name="PPHeaderTop" xfId="2" xr:uid="{0275E807-2B3F-44C3-B981-CC3CC045D5B5}"/>
+    <cellStyle name="PPInvalidValue" xfId="6" xr:uid="{C9CA6567-2FF0-4465-9CD7-07AEF0207FFD}"/>
+    <cellStyle name="PPMissingValue" xfId="7" xr:uid="{A89BB8C0-0843-42CF-95F5-9C49C5C6766B}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -275,6 +344,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -310,6 +396,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -485,24 +588,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:CA2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="30.7109375" customWidth="1"/>
     <col min="3" max="3" width="30.28515625" customWidth="1"/>
-    <col min="4" max="4" width="31.28515625" customWidth="1"/>
-    <col min="5" max="5" width="30.42578125" customWidth="1"/>
-    <col min="6" max="6" width="30.85546875" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" customWidth="1"/>
-    <col min="9" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="10" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="39.28515625" customWidth="1"/>
+    <col min="5" max="5" width="31.28515625" customWidth="1"/>
+    <col min="6" max="6" width="30.42578125" customWidth="1"/>
+    <col min="7" max="7" width="30.85546875" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" customWidth="1"/>
     <col min="11" max="11" width="15.7109375" customWidth="1"/>
-    <col min="12" max="12" width="16.7109375" customWidth="1"/>
-    <col min="13" max="13" width="72.42578125" style="8" customWidth="1"/>
-    <col min="14" max="50" width="11.5703125" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" customWidth="1"/>
+    <col min="13" max="13" width="15.7109375" customWidth="1"/>
+    <col min="14" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="50" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:79" s="4" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -516,40 +620,40 @@
         <v>9</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>13</v>
       </c>
       <c r="P1" s="4" t="s">
         <v>13</v>
@@ -745,10 +849,10 @@
       </c>
     </row>
     <row r="2" spans="1:79" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="7"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -757,14 +861,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="30.7109375" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
@@ -780,8 +885,14 @@
       <c r="E1" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C2" s="1"/>
     </row>
   </sheetData>
@@ -791,6 +902,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <documentManagement>
     <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
@@ -803,7 +923,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -906,16 +1026,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE4C072F-EAF4-499E-9347-564ED0FAEA38}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE9C6564-CDD5-499C-B8DC-E1612B398E0A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -932,7 +1051,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{020D619E-1B83-458E-AA82-82A7D933447F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -949,12 +1068,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE4C072F-EAF4-499E-9347-564ED0FAEA38}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Revert "Merged PR 263: 4951 - Update Resource Type Import/Export for MOQ Types
4951 - Update Resource Type Import/Export for MOQ Types"
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Tests/ActionLogic/Export/LaborTypesAndSpread.xlsx
+++ b/GenBOE/GenBOE.Tests/ActionLogic/Export/LaborTypesAndSpread.xlsx
@@ -1,26 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22527"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\Git\genboe\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF5D9862-E213-4160-AAFC-BCBA56549906}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="90" windowWidth="19320" windowHeight="11760"/>
   </bookViews>
   <sheets>
     <sheet name="Labor Types" sheetId="3" r:id="rId1"/>
     <sheet name="Options Lists" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="CLINs">'Options Lists'!$E$2</definedName>
+    <definedName name="Clins">'Options Lists'!$E$2</definedName>
     <definedName name="COST_STYLE">#REF!</definedName>
-    <definedName name="MOQTypes">'Options Lists'!$G$2</definedName>
-    <definedName name="Offload">'Options Lists'!$F$2</definedName>
     <definedName name="PerfOrgs">'Options Lists'!$B$2</definedName>
     <definedName name="Resources">'Options Lists'!$A$2</definedName>
     <definedName name="SpreadCurves">'Options Lists'!$C$2</definedName>
@@ -31,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="19">
   <si>
     <t>Performing Orgs</t>
   </si>
@@ -87,23 +84,18 @@
     <t>CLIN</t>
   </si>
   <si>
-    <t>Offload</t>
-  </si>
-  <si>
-    <t>MOQ Type</t>
-  </si>
-  <si>
-    <t>MOQTypes</t>
+    <t>Reference</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="m/yyyy"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,36 +118,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFECF0F1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFECF0F1"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF452DB2"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -171,36 +135,6 @@
           <color theme="0" tint="-0.25098422193060094"/>
         </stop>
       </gradientFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF070729"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF9F9F9F"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF452DB2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD35714"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -223,19 +157,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="8">
+  <cellStyleXfs count="2">
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="0"/>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="0"/>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="0"/>
-    <xf numFmtId="49" fontId="3" fillId="5" borderId="0"/>
-    <xf numFmtId="49" fontId="3" fillId="6" borderId="0"/>
-    <xf numFmtId="49" fontId="6" fillId="7" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -243,17 +171,20 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="8">
-    <cellStyle name="genBOE" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+  <cellStyles count="2">
+    <cellStyle name="genBOE" xfId="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
-    <cellStyle name="PPDuplicateRow" xfId="5" xr:uid="{9122EC09-67FD-49C5-95A4-2D9419B3FEE0}"/>
-    <cellStyle name="PPHeaderColumn" xfId="3" xr:uid="{37FD2640-2E85-4306-88DE-A00E421F402E}"/>
-    <cellStyle name="PPHeaderRequired" xfId="4" xr:uid="{180094FB-4A1F-402E-8045-8F1F9F48FF85}"/>
-    <cellStyle name="PPHeaderTop" xfId="2" xr:uid="{0275E807-2B3F-44C3-B981-CC3CC045D5B5}"/>
-    <cellStyle name="PPInvalidValue" xfId="6" xr:uid="{C9CA6567-2FF0-4465-9CD7-07AEF0207FFD}"/>
-    <cellStyle name="PPMissingValue" xfId="7" xr:uid="{A89BB8C0-0843-42CF-95F5-9C49C5C6766B}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -344,23 +275,6 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -396,23 +310,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -588,25 +485,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:CA2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="30.7109375" customWidth="1"/>
     <col min="3" max="3" width="30.28515625" customWidth="1"/>
-    <col min="4" max="4" width="39.28515625" customWidth="1"/>
-    <col min="5" max="5" width="31.28515625" customWidth="1"/>
-    <col min="6" max="6" width="30.42578125" customWidth="1"/>
-    <col min="7" max="7" width="30.85546875" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" customWidth="1"/>
-    <col min="9" max="9" width="15.28515625" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" customWidth="1"/>
+    <col min="4" max="4" width="31.28515625" customWidth="1"/>
+    <col min="5" max="5" width="30.42578125" customWidth="1"/>
+    <col min="6" max="6" width="30.85546875" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="8" max="8" width="15.140625" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="10" width="13.42578125" customWidth="1"/>
     <col min="11" max="11" width="15.7109375" customWidth="1"/>
-    <col min="12" max="12" width="13.42578125" customWidth="1"/>
-    <col min="13" max="13" width="15.7109375" customWidth="1"/>
-    <col min="14" max="14" width="16.7109375" customWidth="1"/>
-    <col min="15" max="50" width="11.5703125" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" customWidth="1"/>
+    <col min="13" max="13" width="72.42578125" style="8" customWidth="1"/>
+    <col min="14" max="50" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:79" s="4" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -620,40 +516,40 @@
         <v>9</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="H1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>5</v>
-      </c>
       <c r="N1" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P1" s="4" t="s">
         <v>13</v>
@@ -849,10 +745,10 @@
       </c>
     </row>
     <row r="2" spans="1:79" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -861,15 +757,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="30.7109375" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
@@ -885,14 +780,8 @@
       <c r="E1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>20</v>
-      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C2" s="1"/>
     </row>
   </sheetData>
@@ -902,15 +791,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <documentManagement>
     <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
@@ -923,7 +803,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -1026,15 +906,16 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE4C072F-EAF4-499E-9347-564ED0FAEA38}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE9C6564-CDD5-499C-B8DC-E1612B398E0A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -1051,7 +932,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{020D619E-1B83-458E-AA82-82A7D933447F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1068,4 +949,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE4C072F-EAF4-499E-9347-564ED0FAEA38}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>